<commit_message>
Ändrat massa efter labb (ff lite fel)
</commit_message>
<xml_diff>
--- a/Apriori mapp/apriori_results.xlsx
+++ b/Apriori mapp/apriori_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,10 +444,20 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>Leverage</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Leverage count</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Rule length</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Support count</t>
         </is>
@@ -456,169 +466,363 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SMS conversation O-S-H=verymanysmsconv_O-S-H
-AND SMS received O-S-H=verymanysmsrec_O-S-H</t>
+          <t>BT_Outsiders S-H=manybtout_S-H
+ AND BT_Unique people O-S-H=manybtunq_O-S-H
+ AND SMS sent O-S-H=manysmssent_O-S-H</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SMS sent O-S-H=verymanysmssent_O-S-H</t>
+          <t>BT_Interactions O-S-H=manybtint_O-S-H
+ AND SMS received O-S-H=manysmsrec_O-S-H</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.1026785714285714</v>
+        <v>0.05208333333333334</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9452054794520547</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="E2" t="n">
-        <v>7.3857916533928</v>
+        <v>10.18181818181818</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>0.04696800595238095</v>
       </c>
       <c r="G2" t="n">
-        <v>69</v>
+        <v>32</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SMS sent O-S-H=verymanysmssent_O-S-H</t>
+          <t>BT_Interactions O-S-H=manybtint_O-S-H
+ AND SMS received O-S-H=manysmsrec_O-S-H</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SMS conversation O-S-H=verymanysmsconv_O-S-H
-AND SMS received O-S-H=verymanysmsrec_O-S-H</t>
+          <t>BT_Outsiders S-H=manybtout_S-H
+ AND BT_Unique people O-S-H=manybtunq_O-S-H
+ AND SMS sent O-S-H=manysmssent_O-S-H</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1026785714285714</v>
+        <v>0.05208333333333334</v>
       </c>
       <c r="D3" t="n">
-        <v>0.8023255813953488</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="E3" t="n">
-        <v>7.3857916533928</v>
+        <v>10.18181818181818</v>
       </c>
       <c r="F3" t="n">
-        <v>3</v>
+        <v>0.04696800595238095</v>
       </c>
       <c r="G3" t="n">
-        <v>69</v>
+        <v>32</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SMS conversation O-S-H=verymanysmsconv_O-S-H
-AND SMS sent O-S-H=verymanysmssent_O-S-H</t>
+          <t>BT_Outsiders S-H=manybtout_S-H
+ AND BT_Unique people O-S-H=manybtunq_O-S-H
+ AND SMS received O-S-H=manysmsrec_O-S-H</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SMS received O-S-H=verymanysmsrec_O-S-H</t>
+          <t>BT_Interactions O-S-H=manybtint_O-S-H
+ AND SMS sent O-S-H=manysmssent_O-S-H</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.1026785714285714</v>
+        <v>0.05208333333333334</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9583333333333334</v>
+        <v>0.9210526315789475</v>
       </c>
       <c r="E4" t="n">
-        <v>7.318181818181818</v>
+        <v>10.14667817083693</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>0.04695029053287982</v>
       </c>
       <c r="G4" t="n">
-        <v>69</v>
+        <v>32</v>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SMS received O-S-H=verymanysmsrec_O-S-H</t>
+          <t>BT_Interactions O-S-H=manybtint_O-S-H
+ AND SMS sent O-S-H=manysmssent_O-S-H</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SMS conversation O-S-H=verymanysmsconv_O-S-H
-AND SMS sent O-S-H=verymanysmssent_O-S-H</t>
+          <t>BT_Outsiders S-H=manybtout_S-H
+ AND BT_Unique people O-S-H=manybtunq_O-S-H
+ AND SMS received O-S-H=manysmsrec_O-S-H</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.1026785714285714</v>
+        <v>0.05208333333333334</v>
       </c>
       <c r="D5" t="n">
-        <v>0.7840909090909091</v>
+        <v>0.5737704918032788</v>
       </c>
       <c r="E5" t="n">
-        <v>7.318181818181818</v>
+        <v>10.14667817083693</v>
       </c>
       <c r="F5" t="n">
-        <v>3</v>
+        <v>0.04695029053287982</v>
       </c>
       <c r="G5" t="n">
-        <v>69</v>
+        <v>32</v>
+      </c>
+      <c r="H5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SMS received O-S-H=verymanysmsrec_O-S-H
-AND SMS sent O-S-H=verymanysmssent_O-S-H</t>
+          <t>BT_Unique people O-S-H=manybtunq_O-S-H
+ AND SMS conversation O-S-H=manysmsconv_O-S-H
+ AND SMS received O-S-H=manysmsrec_O-S-H</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SMS conversation O-S-H=verymanysmsconv_O-S-H</t>
+          <t>BT_Average Duration O-S-H=middlebtavgdur_O-S-H
+ AND BT_Interactions O-S-H=manybtint_O-S-H
+ AND SMS sent O-S-H=manysmssent_O-S-H</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.1026785714285714</v>
+        <v>0.0505952380952381</v>
       </c>
       <c r="D6" t="n">
-        <v>0.8518518518518519</v>
+        <v>0.6538461538461539</v>
       </c>
       <c r="E6" t="n">
-        <v>6.360493827160494</v>
+        <v>9.764102564102565</v>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>0.04541347789115646</v>
       </c>
       <c r="G6" t="n">
-        <v>69</v>
+        <v>31</v>
+      </c>
+      <c r="H6" t="n">
+        <v>6</v>
+      </c>
+      <c r="I6" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SMS conversation O-S-H=verymanysmsconv_O-S-H</t>
+          <t>BT_Average Duration O-S-H=middlebtavgdur_O-S-H
+ AND BT_Interactions O-S-H=manybtint_O-S-H
+ AND SMS sent O-S-H=manysmssent_O-S-H</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SMS received O-S-H=verymanysmsrec_O-S-H
-AND SMS sent O-S-H=verymanysmssent_O-S-H</t>
+          <t>BT_Unique people O-S-H=manybtunq_O-S-H
+ AND SMS conversation O-S-H=manysmsconv_O-S-H
+ AND SMS received O-S-H=manysmsrec_O-S-H</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.1026785714285714</v>
+        <v>0.0505952380952381</v>
       </c>
       <c r="D7" t="n">
-        <v>0.7666666666666666</v>
+        <v>0.7555555555555555</v>
       </c>
       <c r="E7" t="n">
-        <v>6.360493827160493</v>
+        <v>9.764102564102563</v>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>0.04541347789115646</v>
       </c>
       <c r="G7" t="n">
-        <v>69</v>
+        <v>31</v>
+      </c>
+      <c r="H7" t="n">
+        <v>6</v>
+      </c>
+      <c r="I7" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BT_Average Duration O-S-H=middlebtavgdur_O-S-H
+ AND BT_Interactions O-S-H=manybtint_O-S-H
+ AND SMS received O-S-H=manysmsrec_O-S-H</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BT_Unique people O-S-H=manybtunq_O-S-H
+ AND SMS conversation O-S-H=manysmsconv_O-S-H
+ AND SMS sent O-S-H=manysmssent_O-S-H</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.0505952380952381</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.8500000000000001</v>
+      </c>
+      <c r="E8" t="n">
+        <v>9.681355932203392</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.04536918934240363</v>
+      </c>
+      <c r="G8" t="n">
+        <v>30</v>
+      </c>
+      <c r="H8" t="n">
+        <v>6</v>
+      </c>
+      <c r="I8" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BT_Unique people O-S-H=manybtunq_O-S-H
+ AND SMS conversation O-S-H=manysmsconv_O-S-H
+ AND SMS sent O-S-H=manysmssent_O-S-H</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BT_Average Duration O-S-H=middlebtavgdur_O-S-H
+ AND BT_Interactions O-S-H=manybtint_O-S-H
+ AND SMS received O-S-H=manysmsrec_O-S-H</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.0505952380952381</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.576271186440678</v>
+      </c>
+      <c r="E9" t="n">
+        <v>9.68135593220339</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.04536918934240363</v>
+      </c>
+      <c r="G9" t="n">
+        <v>30</v>
+      </c>
+      <c r="H9" t="n">
+        <v>6</v>
+      </c>
+      <c r="I9" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>BT_Unique people O-S-H=manybtunq_O-S-H
+ AND SMS received S-H=manysmsrec_S-H</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SMS conversation S-H=manysmsconv_S-H
+ AND SMS sent S-H=manysmssent_S-H</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.0505952380952381</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.8500000000000001</v>
+      </c>
+      <c r="E10" t="n">
+        <v>9.520000000000001</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.04528061224489796</v>
+      </c>
+      <c r="G10" t="n">
+        <v>30</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I10" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SMS conversation S-H=manysmsconv_S-H
+ AND SMS sent S-H=manysmssent_S-H</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>BT_Unique people O-S-H=manybtunq_O-S-H
+ AND SMS received S-H=manysmsrec_S-H</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.0505952380952381</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.5666666666666667</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9.52</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.04528061224489796</v>
+      </c>
+      <c r="G11" t="n">
+        <v>30</v>
+      </c>
+      <c r="H11" t="n">
+        <v>4</v>
+      </c>
+      <c r="I11" t="n">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>